<commit_message>
Create a test case covering education and certificate feature in Mars Project
</commit_message>
<xml_diff>
--- a/TA_Mars_Test Cases.xlsx
+++ b/TA_Mars_Test Cases.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\Desktop\Future job preparation content\Internship Main Task Folder\Task1_Project\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\Desktop\Future job preparation content\Internship Main Task Folder\Task1_Project\On-Boarding-Internship-Task\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{07ADAF0E-AE95-4FB7-9903-049EDE4DA289}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2C31F52D-FDEB-405F-A03C-35FC98BEF70A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{79221562-EBBE-44A3-8DD9-D094D4CE996C}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="44">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="133" uniqueCount="117">
   <si>
     <t>Test Scenario ID</t>
   </si>
@@ -517,6 +517,285 @@
   </si>
   <si>
     <t>TS_S004</t>
+  </si>
+  <si>
+    <t>Write Test Scenarios and Cases for Project Mars (for education section) (task 3)</t>
+  </si>
+  <si>
+    <t>1. Validate that the user can successfully add a new education record by entering all mandatory fields (Country, University, Title, Degree, Graduation Year).</t>
+  </si>
+  <si>
+    <t>TS_E001</t>
+  </si>
+  <si>
+    <t>Validate that the user can add a new education record with all mandatory fields.</t>
+  </si>
+  <si>
+    <t>3. Validate that the system displays a “Duplicate data is not allowed” notification when the user adds a record with the same University, Title, and Degree (even if the graduation year differs).</t>
+  </si>
+  <si>
+    <t>4. Validate that the user can add another record with the same University and Title but a different Degree (should be allowed).</t>
+  </si>
+  <si>
+    <t>5. Validate that the user can add multiple education records (no restriction on number of entries).</t>
+  </si>
+  <si>
+    <t>6. Validate that clicking the “Cancel” button while adding a new education record discards all entered data and closes the form.</t>
+  </si>
+  <si>
+    <t>7. Validate that after adding a new education record, a success notification appears.</t>
+  </si>
+  <si>
+    <t>8. Validate that the added data persists after page refresh or re-login.</t>
+  </si>
+  <si>
+    <t>9. Validate the character limit for each field (e.g., University name or Degree field should not exceed expected limits).</t>
+  </si>
+  <si>
+    <t>10. Validate that special characters (e.g., !@#$%) are not accepted in the University, Title, or Degree fields.</t>
+  </si>
+  <si>
+    <t>11. Validate system behavior when an extremely large payload is submitted — for example, pasting a 10,000-character string into the “University” field to test robustness.</t>
+  </si>
+  <si>
+    <t>12. Validate that the system remains stable (no crash or timeout) when multiple education records are added continuously without page refresh.</t>
+  </si>
+  <si>
+    <t>2. Validate that the system shows an error message when any mandatory field (e.g., University or Degree name) is left blank.</t>
+  </si>
+  <si>
+    <t>TS_E002</t>
+  </si>
+  <si>
+    <t>Validate that the user can edit an existing education record with all mandatory fields.</t>
+  </si>
+  <si>
+    <t>1. Validate that the user can successfully edit an existing education record with all valid inputs (Country, University, Title, Degree, Graduation Year).</t>
+  </si>
+  <si>
+    <t>2. Validate that the system prevents saving when any mandatory field is left blank and displays a proper error message.</t>
+  </si>
+  <si>
+    <t>4. Validate that the system allows editing when the updated data is unique (e.g., changing Degree or Title to a new valid value).</t>
+  </si>
+  <si>
+    <t>5. Validate that after successful editing, a notification appears confirming the update.</t>
+  </si>
+  <si>
+    <t>6. Validate that the updated data is correctly saved and persists after refresh or re-login.</t>
+  </si>
+  <si>
+    <t>7. Validate that entering invalid characters (e.g., !@#$%) in the University, Title, or Degree fields displays an appropriate error message.</t>
+  </si>
+  <si>
+    <t>8. Validate that the user can update only selected fields (e.g., change only Graduation Year) and other existing values remain unchanged.</t>
+  </si>
+  <si>
+    <t>9. Validate that the system handles extremely long text input in fields (e.g., pasting 10,000 characters in University name) without crashing.</t>
+  </si>
+  <si>
+    <t>3. Validate that the system shows “information already exists” when edited data matches an existing record (same University, Title, and Degree).</t>
+  </si>
+  <si>
+    <t>10. Validate that quickly editing and saving the same record multiple times does not cause data corruption or system errors.</t>
+  </si>
+  <si>
+    <t>TS_E003</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Validate that the user can delete an existing education record. </t>
+  </si>
+  <si>
+    <t>TS_E004</t>
+  </si>
+  <si>
+    <t>Validate that the user can view the education record.</t>
+  </si>
+  <si>
+    <r>
+      <t>2.</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="7"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t>  </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>Validate that a confirmation pop-up appears before deleting a record.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">1. </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="7"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>Validate that the user can delete an existing education record successfully.</t>
+    </r>
+  </si>
+  <si>
+    <t>3. Validate that the deleted record no longer appears in the list after page refresh or re-login.</t>
+  </si>
+  <si>
+    <t>4. Validate that rapidly clicking the delete button multiple times does not cause system crash or data inconsistency.</t>
+  </si>
+  <si>
+    <t>5. Validate that deleting multiple records back-to-back does not cause performance issues or timeout.</t>
+  </si>
+  <si>
+    <t>1. Validate that all added education records are visible in the user’s profile.</t>
+  </si>
+  <si>
+    <t>2. Validate that each record displays correct details — Country, University, Title, Degree, and Graduation Year.</t>
+  </si>
+  <si>
+    <t>3. Validate that after page refresh or re-login, all education records are still visible and accurate.</t>
+  </si>
+  <si>
+    <t>4. Validate that viewing a large number of education records does not cause UI lag, crash, or incomplete loading.</t>
+  </si>
+  <si>
+    <t>Write Test Scenarios and Cases for Project Mars (for Certificate section) (task 3)</t>
+  </si>
+  <si>
+    <t>TS_C001</t>
+  </si>
+  <si>
+    <t>TS_C002</t>
+  </si>
+  <si>
+    <t>TS_C003</t>
+  </si>
+  <si>
+    <t>TS_C004</t>
+  </si>
+  <si>
+    <t>Validate that the user can add a new certificate record with all mandatory fields.</t>
+  </si>
+  <si>
+    <t>Validate that the user can edit an existing certificate record with all mandatory fields.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Validate that the user can delete an existing certificate record. </t>
+  </si>
+  <si>
+    <t>Validate that the user can view the certificate record.</t>
+  </si>
+  <si>
+    <t>1. Validate that the user can successfully add a new certificate/award record with all mandatory fields (Certificate/Award, Certificate From, Year).</t>
+  </si>
+  <si>
+    <t>2. Validate that the system shows an error message when any mandatory field is left blank.</t>
+  </si>
+  <si>
+    <t>3. Validate that the system displays “Duplicate data is not allowed” when the user adds a record with the same Certificate/Award and Certificate From (even if the year differs).</t>
+  </si>
+  <si>
+    <t>4. Validate that adding another record with the same Certificate/Award but a different “Certificate From” is allowed.</t>
+  </si>
+  <si>
+    <t>5. Validate that the user can add multiple certificate records (no restriction on number of entries).</t>
+  </si>
+  <si>
+    <t>6. Validate that clicking “Cancel” while adding a new certificate discards input and closes the form.</t>
+  </si>
+  <si>
+    <t>7. Validate that after adding a new certificate, a success notification appears.</t>
+  </si>
+  <si>
+    <t>8. Validate that the added certificate data persists after page refresh or re-login.</t>
+  </si>
+  <si>
+    <t>9. Validate that invalid characters (e.g., !@#$%) in Certificate/Award or Certificate From are handled.</t>
+  </si>
+  <si>
+    <t>10. Validate that pasting a very large text (e.g., 10,000 characters) in Certificate/Award or Certificate From does not crash the system.</t>
+  </si>
+  <si>
+    <t>12. Validate that rapidly adding multiple certificates does not cause performance issues or timeouts.</t>
+  </si>
+  <si>
+    <t>11. Validate the character limit for each field (e.g.Certificate/Award, Certificate From field should not exceed expected limits).</t>
+  </si>
+  <si>
+    <t>1. Validate that the user can successfully edit an existing certificate record with all valid inputs (Certificate/Award, Certificate From, Year).</t>
+  </si>
+  <si>
+    <t>3. Validate that the system shows “duplicate data” when edited data matches an existing record (same Certificate/Award, Certificate From,).</t>
+  </si>
+  <si>
+    <t>4. Validate that the system allows editing when the updated data is unique (e.g., changing Certificate/Award or Certificate From, to a new valid value).</t>
+  </si>
+  <si>
+    <t>7. Validate that entering invalid characters (e.g., !@#$%) in the Certificate/Award or Certificate From fields displays an appropriate error message.</t>
+  </si>
+  <si>
+    <t>8. Validate that the user can update only selected fields (e.g., change only Year) and other existing values remain unchanged.</t>
+  </si>
+  <si>
+    <t>9. Validate that the system handles extremely long text input in fields (e.g., pasting 10,000 characters in Certificate/Award or Certificate From) without crashing.</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">1. </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="7"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>Validate that the user can delete an existing certificate record successfully.</t>
+    </r>
+  </si>
+  <si>
+    <t>2. Validate that each record displays correct details — Certificate/Award, Certificate From, and Year.</t>
+  </si>
+  <si>
+    <t>4. Validate that rapidly clicking the delete button multiple times does not cause a system crash or data inconsistency.</t>
+  </si>
+  <si>
+    <t>1. Validate that all added Certificate records are visible in the user’s profile.</t>
+  </si>
+  <si>
+    <t>3. Validate that after page refresh or re-login, all Certificate records are still visible and accurate.</t>
+  </si>
+  <si>
+    <t>4. Validate that viewing a large number of Certificate records does not cause UI lag, crash, or incomplete loading.</t>
   </si>
 </sst>
 </file>
@@ -578,7 +857,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -591,20 +870,19 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -919,7 +1197,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2E961854-839D-4490-BDB3-772432EA2C88}">
-  <dimension ref="A1:C42"/>
+  <dimension ref="A1:C114"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="28.21875" customWidth="1"/>
@@ -939,7 +1217,7 @@
       </c>
     </row>
     <row r="2" spans="1:3" ht="17.399999999999999" x14ac:dyDescent="0.3">
-      <c r="A2" s="11" t="s">
+      <c r="A2" s="7" t="s">
         <v>35</v>
       </c>
       <c r="B2" s="8"/>
@@ -1003,25 +1281,21 @@
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="B13" s="6"/>
       <c r="C13" s="4" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="14" spans="1:3" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B14" s="6"/>
       <c r="C14" s="4" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="B15" s="6"/>
       <c r="C15" s="4" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="B16" s="6"/>
       <c r="C16" s="3" t="s">
         <v>17</v>
       </c>
@@ -1054,21 +1328,21 @@
       <c r="B22" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="C22" s="7" t="s">
+      <c r="C22" s="6" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A23" s="5"/>
       <c r="B23" s="3"/>
-      <c r="C23" s="7"/>
+      <c r="C23" s="6"/>
     </row>
     <row r="24" spans="1:3" ht="17.399999999999999" x14ac:dyDescent="0.3">
-      <c r="A24" s="10" t="s">
+      <c r="A24" s="9" t="s">
         <v>24</v>
       </c>
-      <c r="B24" s="9"/>
-      <c r="C24" s="9"/>
+      <c r="B24" s="10"/>
+      <c r="C24" s="10"/>
     </row>
     <row r="25" spans="1:3" ht="28.2" x14ac:dyDescent="0.3">
       <c r="A25" s="5" t="s">
@@ -1169,10 +1443,393 @@
         <v>34</v>
       </c>
     </row>
+    <row r="44" spans="1:3" ht="17.399999999999999" x14ac:dyDescent="0.3">
+      <c r="A44" s="9" t="s">
+        <v>44</v>
+      </c>
+      <c r="B44" s="10"/>
+      <c r="C44" s="10"/>
+    </row>
+    <row r="45" spans="1:3" ht="28.2" x14ac:dyDescent="0.3">
+      <c r="A45" s="5" t="s">
+        <v>46</v>
+      </c>
+      <c r="B45" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="C45" s="4" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="46" spans="1:3" ht="27.6" x14ac:dyDescent="0.3">
+      <c r="C46" s="4" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="47" spans="1:3" ht="27.6" x14ac:dyDescent="0.3">
+      <c r="C47" s="4" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="48" spans="1:3" ht="27.6" x14ac:dyDescent="0.3">
+      <c r="C48" s="4" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="49" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="C49" s="4" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="50" spans="1:3" ht="27.6" x14ac:dyDescent="0.3">
+      <c r="C50" s="4" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="51" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="C51" s="4" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="52" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="C52" s="3" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="53" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="C53" s="4" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="54" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="C54" s="4" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="55" spans="1:3" ht="27.6" x14ac:dyDescent="0.3">
+      <c r="C55" s="4" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="56" spans="1:3" ht="28.2" x14ac:dyDescent="0.3">
+      <c r="C56" s="3" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="58" spans="1:3" ht="28.2" x14ac:dyDescent="0.3">
+      <c r="A58" s="5" t="s">
+        <v>59</v>
+      </c>
+      <c r="B58" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="C58" s="4" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="59" spans="1:3" ht="27.6" x14ac:dyDescent="0.3">
+      <c r="C59" s="4" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="60" spans="1:3" ht="27.6" x14ac:dyDescent="0.3">
+      <c r="C60" s="4" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="61" spans="1:3" ht="27.6" x14ac:dyDescent="0.3">
+      <c r="C61" s="4" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="62" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="C62" s="4" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="63" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="C63" s="4" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="64" spans="1:3" ht="27.6" x14ac:dyDescent="0.3">
+      <c r="C64" s="4" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="65" spans="1:3" ht="28.2" x14ac:dyDescent="0.3">
+      <c r="C65" s="3" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="66" spans="1:3" ht="27.6" x14ac:dyDescent="0.3">
+      <c r="C66" s="4" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="67" spans="1:3" ht="27.6" x14ac:dyDescent="0.3">
+      <c r="C67" s="4" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="68" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="C68" s="4"/>
+    </row>
+    <row r="69" spans="1:3" ht="28.2" x14ac:dyDescent="0.3">
+      <c r="A69" s="5" t="s">
+        <v>71</v>
+      </c>
+      <c r="B69" s="3" t="s">
+        <v>72</v>
+      </c>
+      <c r="C69" s="4" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="70" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="C70" s="4" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="71" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="C71" s="3" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="72" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="C72" s="4" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="73" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="C73" s="4" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="75" spans="1:3" ht="28.2" x14ac:dyDescent="0.3">
+      <c r="A75" s="5" t="s">
+        <v>73</v>
+      </c>
+      <c r="B75" s="3" t="s">
+        <v>74</v>
+      </c>
+      <c r="C75" s="6" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="76" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="C76" s="2" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="77" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="C77" s="2" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="78" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="C78" s="2" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="79" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="C79" s="2"/>
+    </row>
+    <row r="80" spans="1:3" ht="17.399999999999999" x14ac:dyDescent="0.3">
+      <c r="A80" s="9" t="s">
+        <v>84</v>
+      </c>
+      <c r="B80" s="10"/>
+      <c r="C80" s="10"/>
+    </row>
+    <row r="81" spans="1:3" ht="28.2" x14ac:dyDescent="0.3">
+      <c r="A81" s="5" t="s">
+        <v>85</v>
+      </c>
+      <c r="B81" s="3" t="s">
+        <v>89</v>
+      </c>
+      <c r="C81" s="4" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="82" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="C82" s="4" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="83" spans="1:3" ht="27.6" x14ac:dyDescent="0.3">
+      <c r="C83" s="4" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="84" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="C84" s="4" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="85" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="C85" s="4" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="86" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="C86" s="4" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="87" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="C87" s="4" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="88" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="C88" s="3" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="89" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="C89" s="4" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="90" spans="1:3" ht="27.6" x14ac:dyDescent="0.3">
+      <c r="C90" s="4" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="91" spans="1:3" ht="27.6" x14ac:dyDescent="0.3">
+      <c r="C91" s="4" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="92" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="C92" s="3" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="94" spans="1:3" ht="28.2" x14ac:dyDescent="0.3">
+      <c r="A94" s="5" t="s">
+        <v>86</v>
+      </c>
+      <c r="B94" s="3" t="s">
+        <v>90</v>
+      </c>
+      <c r="C94" s="4" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="95" spans="1:3" ht="27.6" x14ac:dyDescent="0.3">
+      <c r="C95" s="4" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="96" spans="1:3" ht="27.6" x14ac:dyDescent="0.3">
+      <c r="C96" s="4" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="97" spans="1:3" ht="27.6" x14ac:dyDescent="0.3">
+      <c r="C97" s="4" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="98" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="C98" s="4" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="99" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="C99" s="4" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="100" spans="1:3" ht="27.6" x14ac:dyDescent="0.3">
+      <c r="C100" s="4" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="101" spans="1:3" ht="28.2" x14ac:dyDescent="0.3">
+      <c r="C101" s="3" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="102" spans="1:3" ht="27.6" x14ac:dyDescent="0.3">
+      <c r="C102" s="4" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="103" spans="1:3" ht="27.6" x14ac:dyDescent="0.3">
+      <c r="C103" s="4" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="104" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="C104" s="4"/>
+    </row>
+    <row r="105" spans="1:3" ht="28.2" x14ac:dyDescent="0.3">
+      <c r="A105" s="5" t="s">
+        <v>87</v>
+      </c>
+      <c r="B105" s="3" t="s">
+        <v>91</v>
+      </c>
+      <c r="C105" s="4" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="106" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="C106" s="4" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="107" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="C107" s="3" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="108" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="C108" s="4" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="109" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="C109" s="4" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="111" spans="1:3" ht="28.2" x14ac:dyDescent="0.3">
+      <c r="A111" s="5" t="s">
+        <v>88</v>
+      </c>
+      <c r="B111" s="3" t="s">
+        <v>92</v>
+      </c>
+      <c r="C111" s="6" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="112" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="C112" s="2" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="113" spans="3:3" x14ac:dyDescent="0.3">
+      <c r="C113" s="2" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="114" spans="3:3" x14ac:dyDescent="0.3">
+      <c r="C114" s="2" t="s">
+        <v>116</v>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="2">
+  <mergeCells count="4">
     <mergeCell ref="A2:C2"/>
     <mergeCell ref="A24:C24"/>
+    <mergeCell ref="A44:C44"/>
+    <mergeCell ref="A80:C80"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>